<commit_message>
Update Test QA - PT. Pranala Ragam Karya.xlsx
</commit_message>
<xml_diff>
--- a/Test QA - PT. Pranala Ragam Karya.xlsx
+++ b/Test QA - PT. Pranala Ragam Karya.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adaml\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TEST QA\Test-QA---PT.-Pranala-Ragam-Karya\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56747B4D-8379-4071-A699-6EE9E52B5C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24925E6C-3142-46A5-B068-920332828EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B2FFC2E4-2BB6-40B3-94BA-7BC27872A5F3}"/>
   </bookViews>
@@ -260,9 +260,6 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -277,6 +274,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,219 +604,219 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>2</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>3</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>4</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>5</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="1"/>
+      <c r="B10" s="6"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>1</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="105" x14ac:dyDescent="0.25">
-      <c r="B14" s="4">
+      <c r="B14" s="3">
         <v>2</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <v>3</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="B16" s="4">
+      <c r="B16" s="3">
         <v>4</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="B17" s="4">
+      <c r="B17" s="3">
         <v>5</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="5" t="s">
         <v>50</v>
       </c>
     </row>
@@ -824,16 +824,16 @@
       <c r="A18" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="4">
-        <v>5</v>
-      </c>
-      <c r="C18" s="6" t="s">
+      <c r="B18" s="3">
+        <v>6</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="5" t="s">
         <v>51</v>
       </c>
     </row>
@@ -855,10 +855,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="4">
+      <c r="A1" s="3">
         <v>1</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>